<commit_message>
Updated coal CAPEX values to SK
</commit_message>
<xml_diff>
--- a/InputData/elec/ASCAPEX/Annual Sustaining CAPEX by Generator Age.xlsx
+++ b/InputData/elec/ASCAPEX/Annual Sustaining CAPEX by Generator Age.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASCAPEX-base" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASCAPEX-slope" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASCAPEX-adder30" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASCAPEX-adder40" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="About" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ASCAPEX-base" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ASCAPEX-slope" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ASCAPEX-adder30" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ASCAPEX-adder40" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -573,9 +573,6 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -594,6 +591,18 @@
       <c r="A22" t="inlineStr">
         <is>
           <t>Bases reset to the EIA age-0 values per this sheet's own documented method: nuclear and SMR = 28 x 0.8287 = 23,203.60 $/MW-yr; hard coal / lignite (+CCS variants) = (16.53 + 5.68 x 0.654 fleet FGD share) x 0.921 = 18645.39 $/MW-yr. FGD share is capacity-weighted from CCaMC 'Annual CAPEX Calcs' (565 coal units, 227 GW). SMR note: its old flat constant simply copied aged-fleet nuclear; a new-build tech is set to the age-0 EIA base for consistency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>South Korea update 2026-10-28:</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Coal/lignite (+CCS) base reset to (16.53 + 5.68 x 1.0 FGD share) x 0.921 = 20455.41 $/MW-yr (US value used 0.654). FGD share ~1.0 is a working estimate, partly checked 2026-10-28: KC Cottrell 2008 UN-ESCAP deck (FGD on 30 coal units / 14,565 MW installed 1997-2005); FGD required at all plants from Jan 1999; KEPCO FY2019 Form 20-F plant anti-pollution lists show FGD at Boryeong 3-8, Taean 1-4, Hadong 2-6, Dangjin 1-10, Samcheonpo 5-6, Donghae 1-2. No unit-level census found; Taean 5-10 and Hadong 1, 7-8 are not named in the 20-F lists (not flagged as lacking FGD). Verify against KEPCO gencos / Ministry of Environment unit data. Slopes/adders unchanged. Values are deliberately NOT scaled by the Korea/US construction-cost ratio (0.461): Korean anchors (KEEI 17-16 life-extension at 20% of new build, ~$27/kW-yr; MOTIE 2018 environmental retrofit plan, ~$21/kW-yr) sit near the unscaled ~$23/kW-yr, not the scaled ~$10.5.</t>
         </is>
       </c>
     </row>
@@ -631,7 +640,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>18645.39</v>
+        <v>20455.41</v>
       </c>
     </row>
     <row r="3">
@@ -763,7 +772,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>18645.39</v>
+        <v>20455.41</v>
       </c>
     </row>
     <row r="15">
@@ -817,7 +826,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>18645.39</v>
+        <v>20455.41</v>
       </c>
     </row>
     <row r="20">
@@ -849,7 +858,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>18645.39</v>
+        <v>20455.41</v>
       </c>
     </row>
     <row r="23">

</xml_diff>